<commit_message>
data(jpy): daily refresh 2026-09-14T08:03Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{05C4E2D1-309F-44FB-B53B-C2952139F314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{97FC705E-C89B-42D1-9198-87E418F56492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46275</v>
+        <v>46276</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46275</v>
+        <v>46276</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>129985</v>
+        <v>131320</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23861</v>
+        <v>24132</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>106124</v>
+        <v>107188</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,7 +2582,7 @@
         <v>0.95</v>
       </c>
       <c r="I11" s="36">
-        <v>1.03</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="J11" s="39">
         <v>0.97699999999999998</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M12" s="45" t="s">
-        <v>46</v>
+      <c r="K12" s="43">
+        <v>1.03</v>
+      </c>
+      <c r="L12" s="43">
+        <v>1.03</v>
+      </c>
+      <c r="M12" s="45">
+        <v>1.03</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>40837</v>
+        <v>42491</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2772,14 +2772,14 @@
       <c r="J15" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K15" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L15" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M15" s="54" t="s">
-        <v>46</v>
+      <c r="K15" s="52">
+        <v>1.08</v>
+      </c>
+      <c r="L15" s="52">
+        <v>1.08</v>
+      </c>
+      <c r="M15" s="54">
+        <v>1.08</v>
       </c>
     </row>
     <row r="16" spans="1:19" ht="39.9" customHeight="1">
@@ -2813,14 +2813,14 @@
       <c r="J16" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M16" s="54" t="s">
-        <v>46</v>
+      <c r="K16" s="52">
+        <v>1.08</v>
+      </c>
+      <c r="L16" s="52">
+        <v>1.08</v>
+      </c>
+      <c r="M16" s="54">
+        <v>1.08</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58">
-        <v>1.06</v>
-      </c>
-      <c r="L18" s="58">
-        <v>1.08</v>
-      </c>
-      <c r="M18" s="60">
-        <v>1.07</v>
+      <c r="K18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2936,14 +2936,14 @@
       <c r="J19" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="43">
-        <v>0.98099999999999998</v>
-      </c>
-      <c r="L19" s="43">
-        <v>0.98099999999999998</v>
-      </c>
-      <c r="M19" s="45">
-        <v>0.98099999999999998</v>
+      <c r="K19" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L19" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M19" s="45" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="54" t="s">
-        <v>46</v>
+      <c r="K20" s="52">
+        <v>1.0409999999999999</v>
+      </c>
+      <c r="L20" s="52">
+        <v>1.05</v>
+      </c>
+      <c r="M20" s="54">
+        <v>1.044</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3018,14 +3018,14 @@
       <c r="J21" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M21" s="60" t="s">
-        <v>46</v>
+      <c r="K21" s="58">
+        <v>1.43</v>
+      </c>
+      <c r="L21" s="58">
+        <v>1.43</v>
+      </c>
+      <c r="M21" s="60">
+        <v>1.43</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.27</v>
+        <v>1.38</v>
       </c>
       <c r="L22" s="65">
-        <v>1.35</v>
+        <v>1.38</v>
       </c>
       <c r="M22" s="67">
-        <v>1.292</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3091,14 +3091,14 @@
       <c r="G23" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="52">
-        <v>1.37</v>
-      </c>
-      <c r="I23" s="52">
-        <v>1.37</v>
-      </c>
-      <c r="J23" s="55">
-        <v>1.37</v>
+      <c r="H23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J23" s="55" t="s">
+        <v>46</v>
       </c>
       <c r="K23" s="52" t="s">
         <v>3</v>
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="K24" s="52">
+        <v>1.42</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.42</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.42</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">
@@ -3182,14 +3182,14 @@
       <c r="J25" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K25" s="52">
-        <v>1.575</v>
-      </c>
-      <c r="L25" s="52">
-        <v>1.575</v>
-      </c>
-      <c r="M25" s="54">
-        <v>1.575</v>
+      <c r="K25" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L25" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M25" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-15T07:57Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{97FC705E-C89B-42D1-9198-87E418F56492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{28C61FD4-7E89-4387-A874-A971B2844C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46276</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>131320</v>
+        <v>131714</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>24132</v>
+        <v>23816</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>107188</v>
+        <v>107898</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,7 +2582,7 @@
         <v>0.95</v>
       </c>
       <c r="I11" s="36">
-        <v>0.97799999999999998</v>
+        <v>1.03</v>
       </c>
       <c r="J11" s="39">
         <v>0.97699999999999998</v>
@@ -2634,13 +2634,13 @@
         <v>50</v>
       </c>
       <c r="K12" s="43">
-        <v>1.03</v>
+        <v>1.0249999999999999</v>
       </c>
       <c r="L12" s="43">
-        <v>1.03</v>
+        <v>1.0249999999999999</v>
       </c>
       <c r="M12" s="45">
-        <v>1.03</v>
+        <v>1.0249999999999999</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>42491</v>
+        <v>43211</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2772,14 +2772,14 @@
       <c r="J15" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K15" s="52">
-        <v>1.08</v>
-      </c>
-      <c r="L15" s="52">
-        <v>1.08</v>
-      </c>
-      <c r="M15" s="54">
-        <v>1.08</v>
+      <c r="K15" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L15" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M15" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:19" ht="39.9" customHeight="1">
@@ -2804,23 +2804,23 @@
       <c r="G16" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J16" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="K16" s="52">
-        <v>1.08</v>
-      </c>
-      <c r="L16" s="52">
-        <v>1.08</v>
-      </c>
-      <c r="M16" s="54">
-        <v>1.08</v>
+      <c r="H16" s="52">
+        <v>0.97</v>
+      </c>
+      <c r="I16" s="52">
+        <v>0.97</v>
+      </c>
+      <c r="J16" s="55">
+        <v>0.97</v>
+      </c>
+      <c r="K16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M16" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="39.9" customHeight="1">
@@ -2927,14 +2927,14 @@
       <c r="G19" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="H19" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="I19" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="J19" s="46" t="s">
-        <v>46</v>
+      <c r="H19" s="43">
+        <v>1.0549999999999999</v>
+      </c>
+      <c r="I19" s="43">
+        <v>1.0549999999999999</v>
+      </c>
+      <c r="J19" s="46">
+        <v>1.0549999999999999</v>
       </c>
       <c r="K19" s="43" t="s">
         <v>3</v>
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.0409999999999999</v>
+        <v>1.07</v>
       </c>
       <c r="L20" s="52">
-        <v>1.05</v>
+        <v>1.28</v>
       </c>
       <c r="M20" s="54">
-        <v>1.044</v>
+        <v>1.1120000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3018,14 +3018,14 @@
       <c r="J21" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K21" s="58">
-        <v>1.43</v>
-      </c>
-      <c r="L21" s="58">
-        <v>1.43</v>
-      </c>
-      <c r="M21" s="60">
-        <v>1.43</v>
+      <c r="K21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M21" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65">
-        <v>1.38</v>
-      </c>
-      <c r="L22" s="65">
-        <v>1.38</v>
-      </c>
-      <c r="M22" s="67">
-        <v>1.38</v>
+      <c r="K22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="M22" s="67" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3091,14 +3091,14 @@
       <c r="G23" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J23" s="55" t="s">
-        <v>46</v>
+      <c r="H23" s="52">
+        <v>1.38</v>
+      </c>
+      <c r="I23" s="52">
+        <v>1.38</v>
+      </c>
+      <c r="J23" s="55">
+        <v>1.38</v>
       </c>
       <c r="K23" s="52" t="s">
         <v>3</v>
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52">
-        <v>1.42</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.42</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.42</v>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-16T07:51Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{28C61FD4-7E89-4387-A874-A971B2844C82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{2DC0ED37-B371-43D1-822C-86FD7D8579A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46279</v>
+        <v>46280</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46279</v>
+        <v>46280</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>131714</v>
+        <v>134843</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23816</v>
+        <v>24309</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>107898</v>
+        <v>110534</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2585,7 +2585,7 @@
         <v>1.03</v>
       </c>
       <c r="J11" s="39">
-        <v>0.97699999999999998</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43">
-        <v>1.0249999999999999</v>
-      </c>
-      <c r="L12" s="43">
-        <v>1.0249999999999999</v>
-      </c>
-      <c r="M12" s="45">
-        <v>1.0249999999999999</v>
+      <c r="K12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M12" s="45" t="s">
+        <v>46</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2681,14 +2681,14 @@
       <c r="J13" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="43">
-        <v>0.97499999999999998</v>
-      </c>
-      <c r="L13" s="43">
-        <v>0.97499999999999998</v>
-      </c>
-      <c r="M13" s="45">
-        <v>0.97499999999999998</v>
+      <c r="K13" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L13" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M13" s="45" t="s">
+        <v>46</v>
       </c>
       <c r="O13" s="86" t="s">
         <v>25</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>43211</v>
+        <v>46177</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2731,14 +2731,14 @@
       <c r="J14" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K14" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L14" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M14" s="45" t="s">
-        <v>46</v>
+      <c r="K14" s="43">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="L14" s="43">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M14" s="45">
+        <v>1.1000000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="39.9" customHeight="1">
@@ -2804,14 +2804,14 @@
       <c r="G16" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="52">
-        <v>0.97</v>
-      </c>
-      <c r="I16" s="52">
-        <v>0.97</v>
-      </c>
-      <c r="J16" s="55">
-        <v>0.97</v>
+      <c r="H16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J16" s="55" t="s">
+        <v>46</v>
       </c>
       <c r="K16" s="52" t="s">
         <v>3</v>
@@ -2927,23 +2927,23 @@
       <c r="G19" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="H19" s="43">
-        <v>1.0549999999999999</v>
-      </c>
-      <c r="I19" s="43">
-        <v>1.0549999999999999</v>
-      </c>
-      <c r="J19" s="46">
-        <v>1.0549999999999999</v>
-      </c>
-      <c r="K19" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L19" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M19" s="45" t="s">
-        <v>46</v>
+      <c r="H19" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="I19" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="J19" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="K19" s="43">
+        <v>0.98299999999999998</v>
+      </c>
+      <c r="L19" s="43">
+        <v>1</v>
+      </c>
+      <c r="M19" s="45">
+        <v>0.99399999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.07</v>
+        <v>1.06</v>
       </c>
       <c r="L20" s="52">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="M20" s="54">
-        <v>1.1120000000000001</v>
+        <v>1.083</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3091,23 +3091,23 @@
       <c r="G23" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="52">
-        <v>1.38</v>
-      </c>
-      <c r="I23" s="52">
-        <v>1.38</v>
-      </c>
-      <c r="J23" s="55">
-        <v>1.38</v>
-      </c>
-      <c r="K23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M23" s="54" t="s">
-        <v>46</v>
+      <c r="H23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J23" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="K23" s="52">
+        <v>1.35</v>
+      </c>
+      <c r="L23" s="52">
+        <v>1.39</v>
+      </c>
+      <c r="M23" s="54">
+        <v>1.3839999999999999</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-17T07:55Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{2DC0ED37-B371-43D1-822C-86FD7D8579A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{43E4617F-0EF9-4DEA-8DFE-BB3409A23948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46280</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>134843</v>
+        <v>134782</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>24309</v>
+        <v>24065</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>110534</v>
+        <v>110717</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,10 +2582,10 @@
         <v>0.95</v>
       </c>
       <c r="I11" s="36">
-        <v>1.03</v>
+        <v>1.0249999999999999</v>
       </c>
       <c r="J11" s="39">
-        <v>0.97799999999999998</v>
+        <v>0.97699999999999998</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>46177</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2731,14 +2731,14 @@
       <c r="J14" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K14" s="43">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="L14" s="43">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="M14" s="45">
-        <v>1.1000000000000001</v>
+      <c r="K14" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L14" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M14" s="45" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="39.9" customHeight="1">
@@ -2940,10 +2940,10 @@
         <v>0.98299999999999998</v>
       </c>
       <c r="L19" s="43">
-        <v>1</v>
+        <v>1.1100000000000001</v>
       </c>
       <c r="M19" s="45">
-        <v>0.99399999999999999</v>
+        <v>1.0169999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.06</v>
+        <v>1.49</v>
       </c>
       <c r="L20" s="52">
-        <v>1.25</v>
+        <v>1.49</v>
       </c>
       <c r="M20" s="54">
-        <v>1.083</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3100,14 +3100,14 @@
       <c r="J23" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="52">
-        <v>1.35</v>
-      </c>
-      <c r="L23" s="52">
-        <v>1.39</v>
-      </c>
-      <c r="M23" s="54">
-        <v>1.3839999999999999</v>
+      <c r="K23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M23" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-18T07:33Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{43E4617F-0EF9-4DEA-8DFE-BB3409A23948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{5E050B41-999C-46DD-8ADD-191EC110EB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46281</v>
+        <v>46282</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46281</v>
+        <v>46282</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>134782</v>
+        <v>131250</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>24065</v>
+        <v>23847</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>110717</v>
+        <v>107403</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,7 +2582,7 @@
         <v>0.95</v>
       </c>
       <c r="I11" s="36">
-        <v>1.0249999999999999</v>
+        <v>1.03</v>
       </c>
       <c r="J11" s="39">
         <v>0.97699999999999998</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M12" s="45" t="s">
-        <v>46</v>
+      <c r="K12" s="43">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="L12" s="43">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M12" s="45">
+        <v>1.1000000000000001</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>46290</v>
+        <v>43916</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="60" t="s">
-        <v>46</v>
+      <c r="K18" s="58">
+        <v>1.32</v>
+      </c>
+      <c r="L18" s="58">
+        <v>1.32</v>
+      </c>
+      <c r="M18" s="60">
+        <v>1.32</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2936,14 +2936,14 @@
       <c r="J19" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="43">
-        <v>0.98299999999999998</v>
-      </c>
-      <c r="L19" s="43">
-        <v>1.1100000000000001</v>
-      </c>
-      <c r="M19" s="45">
-        <v>1.0169999999999999</v>
+      <c r="K19" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L19" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M19" s="45" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52">
-        <v>1.49</v>
-      </c>
-      <c r="L20" s="52">
-        <v>1.49</v>
-      </c>
-      <c r="M20" s="54">
-        <v>1.49</v>
+      <c r="K20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="K24" s="52">
+        <v>1.39</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.45</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.42</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-24T07:44Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{5E050B41-999C-46DD-8ADD-191EC110EB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{DBDE57DE-CD00-4224-964A-766075F00446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46282</v>
+        <v>46283</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>131250</v>
+        <v>132180</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23847</v>
+        <v>26030</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>107403</v>
+        <v>106150</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2579,10 +2579,10 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>0.95</v>
+        <v>0.94</v>
       </c>
       <c r="I11" s="36">
-        <v>1.03</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="J11" s="39">
         <v>0.97699999999999998</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="L12" s="43">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="M12" s="45">
-        <v>1.1000000000000001</v>
+      <c r="K12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M12" s="45" t="s">
+        <v>46</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2681,14 +2681,14 @@
       <c r="J13" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L13" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M13" s="45" t="s">
-        <v>46</v>
+      <c r="K13" s="43">
+        <v>1.21</v>
+      </c>
+      <c r="L13" s="43">
+        <v>1.21</v>
+      </c>
+      <c r="M13" s="45">
+        <v>1.21</v>
       </c>
       <c r="O13" s="86" t="s">
         <v>25</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>43916</v>
+        <v>44254</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2854,14 +2854,14 @@
       <c r="J17" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K17" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="54" t="s">
-        <v>46</v>
+      <c r="K17" s="52">
+        <v>1.2250000000000001</v>
+      </c>
+      <c r="L17" s="52">
+        <v>1.2250000000000001</v>
+      </c>
+      <c r="M17" s="54">
+        <v>1.2250000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="39.9" customHeight="1">
@@ -2896,13 +2896,13 @@
         <v>46</v>
       </c>
       <c r="K18" s="58">
-        <v>1.32</v>
+        <v>1.3</v>
       </c>
       <c r="L18" s="58">
-        <v>1.32</v>
+        <v>1.365</v>
       </c>
       <c r="M18" s="60">
-        <v>1.32</v>
+        <v>1.3480000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2936,14 +2936,14 @@
       <c r="J19" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L19" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M19" s="45" t="s">
-        <v>46</v>
+      <c r="K19" s="43">
+        <v>1.226</v>
+      </c>
+      <c r="L19" s="43">
+        <v>1.232</v>
+      </c>
+      <c r="M19" s="45">
+        <v>1.2270000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="54" t="s">
-        <v>46</v>
+      <c r="K20" s="52">
+        <v>1.35</v>
+      </c>
+      <c r="L20" s="52">
+        <v>1.49</v>
+      </c>
+      <c r="M20" s="54">
+        <v>1.42</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="L22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="M22" s="67" t="s">
-        <v>46</v>
+      <c r="K22" s="65">
+        <v>1.35</v>
+      </c>
+      <c r="L22" s="65">
+        <v>1.68</v>
+      </c>
+      <c r="M22" s="67">
+        <v>1.4219999999999999</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52">
-        <v>1.39</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.45</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.42</v>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-25T08:05Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{DBDE57DE-CD00-4224-964A-766075F00446}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{F7242250-AAE3-417D-BFFB-9DC6BD4BE661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46283</v>
+        <v>46289</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46283</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>132180</v>
+        <v>130175</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>26030</v>
+        <v>27127</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>106150</v>
+        <v>103048</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2561,13 +2561,13 @@
         <v>21</v>
       </c>
       <c r="B11" s="35">
-        <v>0.93</v>
+        <v>1.18</v>
       </c>
       <c r="C11" s="36">
-        <v>0.93</v>
+        <v>1.18</v>
       </c>
       <c r="D11" s="36">
-        <v>0.93</v>
+        <v>1.18</v>
       </c>
       <c r="E11" s="37" t="s">
         <v>50</v>
@@ -2579,13 +2579,13 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>0.94</v>
+        <v>1.2</v>
       </c>
       <c r="I11" s="36">
-        <v>0.97799999999999998</v>
+        <v>1.228</v>
       </c>
       <c r="J11" s="39">
-        <v>0.97699999999999998</v>
+        <v>1.2270000000000001</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2681,14 +2681,14 @@
       <c r="J13" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="43">
-        <v>1.21</v>
-      </c>
-      <c r="L13" s="43">
-        <v>1.21</v>
-      </c>
-      <c r="M13" s="45">
-        <v>1.21</v>
+      <c r="K13" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L13" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M13" s="45" t="s">
+        <v>46</v>
       </c>
       <c r="O13" s="86" t="s">
         <v>25</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>44254</v>
+        <v>45888</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2731,14 +2731,14 @@
       <c r="J14" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K14" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L14" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M14" s="45" t="s">
-        <v>46</v>
+      <c r="K14" s="43">
+        <v>1.2</v>
+      </c>
+      <c r="L14" s="43">
+        <v>1.2</v>
+      </c>
+      <c r="M14" s="45">
+        <v>1.2</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="39.9" customHeight="1">
@@ -2855,13 +2855,13 @@
         <v>46</v>
       </c>
       <c r="K17" s="52">
-        <v>1.2250000000000001</v>
+        <v>1.31</v>
       </c>
       <c r="L17" s="52">
-        <v>1.2250000000000001</v>
+        <v>1.37</v>
       </c>
       <c r="M17" s="54">
-        <v>1.2250000000000001</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="39.9" customHeight="1">
@@ -2899,10 +2899,10 @@
         <v>1.3</v>
       </c>
       <c r="L18" s="58">
-        <v>1.365</v>
+        <v>1.3</v>
       </c>
       <c r="M18" s="60">
-        <v>1.3480000000000001</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.226</v>
+        <v>1.5</v>
       </c>
       <c r="L19" s="43">
-        <v>1.232</v>
+        <v>1.5</v>
       </c>
       <c r="M19" s="45">
-        <v>1.2270000000000001</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.35</v>
+        <v>1.31</v>
       </c>
       <c r="L20" s="52">
-        <v>1.49</v>
+        <v>1.47</v>
       </c>
       <c r="M20" s="54">
-        <v>1.42</v>
+        <v>1.3660000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3009,14 +3009,14 @@
       <c r="G21" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="H21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="I21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="J21" s="61" t="s">
-        <v>46</v>
+      <c r="H21" s="58">
+        <v>1.31</v>
+      </c>
+      <c r="I21" s="58">
+        <v>1.31</v>
+      </c>
+      <c r="J21" s="61">
+        <v>1.31</v>
       </c>
       <c r="K21" s="58" t="s">
         <v>3</v>
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.35</v>
+        <v>1.39</v>
       </c>
       <c r="L22" s="65">
-        <v>1.68</v>
+        <v>1.48</v>
       </c>
       <c r="M22" s="67">
-        <v>1.4219999999999999</v>
+        <v>1.413</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3091,14 +3091,14 @@
       <c r="G23" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J23" s="55" t="s">
-        <v>46</v>
+      <c r="H23" s="52">
+        <v>1.38</v>
+      </c>
+      <c r="I23" s="52">
+        <v>1.38</v>
+      </c>
+      <c r="J23" s="55">
+        <v>1.38</v>
       </c>
       <c r="K23" s="52" t="s">
         <v>3</v>
@@ -3132,23 +3132,23 @@
       <c r="G24" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="H24" s="52">
+        <v>1.44</v>
+      </c>
+      <c r="I24" s="52">
+        <v>1.44</v>
+      </c>
+      <c r="J24" s="55">
+        <v>1.44</v>
+      </c>
+      <c r="K24" s="52">
+        <v>1.45</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.48</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.47</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-28T08:53Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{F7242250-AAE3-417D-BFFB-9DC6BD4BE661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{A88B9CA0-F016-43E3-87BB-C3A24BA18061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>130175</v>
+        <v>136883</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>27127</v>
+        <v>23376</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>103048</v>
+        <v>113507</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>45888</v>
+        <v>52322</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2731,14 +2731,14 @@
       <c r="J14" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K14" s="43">
-        <v>1.2</v>
-      </c>
-      <c r="L14" s="43">
-        <v>1.2</v>
-      </c>
-      <c r="M14" s="45">
-        <v>1.2</v>
+      <c r="K14" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L14" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M14" s="45" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="39.9" customHeight="1">
@@ -2854,14 +2854,14 @@
       <c r="J17" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K17" s="52">
-        <v>1.31</v>
-      </c>
-      <c r="L17" s="52">
-        <v>1.37</v>
-      </c>
-      <c r="M17" s="54">
-        <v>1.36</v>
+      <c r="K17" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L17" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M17" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58">
-        <v>1.3</v>
-      </c>
-      <c r="L18" s="58">
-        <v>1.3</v>
-      </c>
-      <c r="M18" s="60">
-        <v>1.3</v>
+      <c r="K18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="L19" s="43">
-        <v>1.5</v>
+        <v>1.52</v>
       </c>
       <c r="M19" s="45">
-        <v>1.5</v>
+        <v>1.304</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52">
-        <v>1.31</v>
-      </c>
-      <c r="L20" s="52">
-        <v>1.47</v>
-      </c>
-      <c r="M20" s="54">
-        <v>1.3660000000000001</v>
+      <c r="K20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3009,23 +3009,23 @@
       <c r="G21" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="H21" s="58">
-        <v>1.31</v>
-      </c>
-      <c r="I21" s="58">
-        <v>1.31</v>
-      </c>
-      <c r="J21" s="61">
-        <v>1.31</v>
-      </c>
-      <c r="K21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M21" s="60" t="s">
-        <v>46</v>
+      <c r="H21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="I21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="J21" s="61" t="s">
+        <v>46</v>
+      </c>
+      <c r="K21" s="58">
+        <v>1.43</v>
+      </c>
+      <c r="L21" s="58">
+        <v>1.43</v>
+      </c>
+      <c r="M21" s="60">
+        <v>1.43</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.39</v>
+        <v>1.36</v>
       </c>
       <c r="L22" s="65">
-        <v>1.48</v>
+        <v>1.5</v>
       </c>
       <c r="M22" s="67">
-        <v>1.413</v>
+        <v>1.407</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3091,23 +3091,23 @@
       <c r="G23" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="52">
-        <v>1.38</v>
-      </c>
-      <c r="I23" s="52">
-        <v>1.38</v>
-      </c>
-      <c r="J23" s="55">
-        <v>1.38</v>
-      </c>
-      <c r="K23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M23" s="54" t="s">
-        <v>46</v>
+      <c r="H23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J23" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="K23" s="52">
+        <v>1.45</v>
+      </c>
+      <c r="L23" s="52">
+        <v>1.49</v>
+      </c>
+      <c r="M23" s="54">
+        <v>1.4830000000000001</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">
@@ -3133,22 +3133,22 @@
         <v>46</v>
       </c>
       <c r="H24" s="52">
-        <v>1.44</v>
+        <v>1.49</v>
       </c>
       <c r="I24" s="52">
-        <v>1.44</v>
+        <v>1.49</v>
       </c>
       <c r="J24" s="55">
-        <v>1.44</v>
-      </c>
-      <c r="K24" s="52">
-        <v>1.45</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.48</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.47</v>
+        <v>1.49</v>
+      </c>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-29T08:52Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{A88B9CA0-F016-43E3-87BB-C3A24BA18061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6827517F-F720-47CF-8967-8930420A3BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46290</v>
+        <v>46293</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46290</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>136883</v>
+        <v>135310</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23376</v>
+        <v>22308</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>113507</v>
+        <v>113002</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2681,14 +2681,14 @@
       <c r="J13" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L13" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M13" s="45" t="s">
-        <v>46</v>
+      <c r="K13" s="43">
+        <v>1.4</v>
+      </c>
+      <c r="L13" s="43">
+        <v>1.4</v>
+      </c>
+      <c r="M13" s="45">
+        <v>1.4</v>
       </c>
       <c r="O13" s="86" t="s">
         <v>25</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>52322</v>
+        <v>53807</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2940,10 +2940,10 @@
         <v>1.2</v>
       </c>
       <c r="L19" s="43">
-        <v>1.52</v>
+        <v>1.22</v>
       </c>
       <c r="M19" s="45">
-        <v>1.304</v>
+        <v>1.21</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="54" t="s">
-        <v>46</v>
+      <c r="K20" s="52">
+        <v>1.2210000000000001</v>
+      </c>
+      <c r="L20" s="52">
+        <v>1.2310000000000001</v>
+      </c>
+      <c r="M20" s="54">
+        <v>1.2270000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3018,14 +3018,14 @@
       <c r="J21" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K21" s="58">
-        <v>1.43</v>
-      </c>
-      <c r="L21" s="58">
-        <v>1.43</v>
-      </c>
-      <c r="M21" s="60">
-        <v>1.43</v>
+      <c r="K21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M21" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.36</v>
+        <v>1.35</v>
       </c>
       <c r="L22" s="65">
-        <v>1.5</v>
+        <v>1.35</v>
       </c>
       <c r="M22" s="67">
-        <v>1.407</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3101,13 +3101,13 @@
         <v>46</v>
       </c>
       <c r="K23" s="52">
-        <v>1.45</v>
+        <v>1.41</v>
       </c>
       <c r="L23" s="52">
-        <v>1.49</v>
+        <v>1.41</v>
       </c>
       <c r="M23" s="54">
-        <v>1.4830000000000001</v>
+        <v>1.41</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">
@@ -3132,23 +3132,23 @@
       <c r="G24" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="52">
+      <c r="H24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="K24" s="52">
         <v>1.49</v>
       </c>
-      <c r="I24" s="52">
+      <c r="L24" s="52">
         <v>1.49</v>
       </c>
-      <c r="J24" s="55">
+      <c r="M24" s="54">
         <v>1.49</v>
-      </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-09-30T08:52Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6827517F-F720-47CF-8967-8930420A3BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{34B63B85-94ED-4CB2-95B5-0EE67905DDEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46293</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>135310</v>
+        <v>136899</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22308</v>
+        <v>22122</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>113002</v>
+        <v>114777</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,7 +2582,7 @@
         <v>1.2</v>
       </c>
       <c r="I11" s="36">
-        <v>1.228</v>
+        <v>1.2290000000000001</v>
       </c>
       <c r="J11" s="39">
         <v>1.2270000000000001</v>
@@ -2681,14 +2681,14 @@
       <c r="J13" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K13" s="43">
-        <v>1.4</v>
-      </c>
-      <c r="L13" s="43">
-        <v>1.4</v>
-      </c>
-      <c r="M13" s="45">
-        <v>1.4</v>
+      <c r="K13" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L13" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M13" s="45" t="s">
+        <v>46</v>
       </c>
       <c r="O13" s="86" t="s">
         <v>25</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>53807</v>
+        <v>55072</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="60" t="s">
-        <v>46</v>
+      <c r="K18" s="58">
+        <v>1.38</v>
+      </c>
+      <c r="L18" s="58">
+        <v>1.38</v>
+      </c>
+      <c r="M18" s="60">
+        <v>1.38</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2940,10 +2940,10 @@
         <v>1.2</v>
       </c>
       <c r="L19" s="43">
-        <v>1.22</v>
+        <v>1.288</v>
       </c>
       <c r="M19" s="45">
-        <v>1.21</v>
+        <v>1.252</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.2210000000000001</v>
+        <v>1.228</v>
       </c>
       <c r="L20" s="52">
-        <v>1.2310000000000001</v>
+        <v>1.4</v>
       </c>
       <c r="M20" s="54">
-        <v>1.2270000000000001</v>
+        <v>1.26</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.35</v>
+        <v>1.29</v>
       </c>
       <c r="L22" s="65">
-        <v>1.35</v>
+        <v>1.38</v>
       </c>
       <c r="M22" s="67">
-        <v>1.35</v>
+        <v>1.3440000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3100,14 +3100,14 @@
       <c r="J23" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="52">
-        <v>1.41</v>
-      </c>
-      <c r="L23" s="52">
-        <v>1.41</v>
-      </c>
-      <c r="M23" s="54">
-        <v>1.41</v>
+      <c r="K23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M23" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52">
-        <v>1.49</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.49</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.49</v>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-01T09:16Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{34B63B85-94ED-4CB2-95B5-0EE67905DDEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{7A3B7AEA-B3E3-4187-8138-5DF472694495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46294</v>
+        <v>46295</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>136899</v>
+        <v>122357</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22122</v>
+        <v>21994</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>114777</v>
+        <v>100363</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2579,13 +2579,13 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>1.2</v>
+        <v>1.19</v>
       </c>
       <c r="I11" s="36">
         <v>1.2290000000000001</v>
       </c>
       <c r="J11" s="39">
-        <v>1.2270000000000001</v>
+        <v>1.226</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M12" s="45" t="s">
-        <v>46</v>
+      <c r="K12" s="43">
+        <v>1.28</v>
+      </c>
+      <c r="L12" s="43">
+        <v>1.38</v>
+      </c>
+      <c r="M12" s="45">
+        <v>1.365</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>55072</v>
+        <v>45179</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2896,13 +2896,13 @@
         <v>46</v>
       </c>
       <c r="K18" s="58">
-        <v>1.38</v>
+        <v>1.2250000000000001</v>
       </c>
       <c r="L18" s="58">
-        <v>1.38</v>
+        <v>1.2250000000000001</v>
       </c>
       <c r="M18" s="60">
-        <v>1.38</v>
+        <v>1.2250000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.2</v>
+        <v>1.22</v>
       </c>
       <c r="L19" s="43">
-        <v>1.288</v>
+        <v>1.232</v>
       </c>
       <c r="M19" s="45">
-        <v>1.252</v>
+        <v>1.2250000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52">
-        <v>1.228</v>
-      </c>
-      <c r="L20" s="52">
-        <v>1.4</v>
-      </c>
-      <c r="M20" s="54">
-        <v>1.26</v>
+      <c r="K20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.29</v>
+        <v>1.24</v>
       </c>
       <c r="L22" s="65">
-        <v>1.38</v>
+        <v>1.37</v>
       </c>
       <c r="M22" s="67">
-        <v>1.3440000000000001</v>
+        <v>1.3320000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3091,14 +3091,14 @@
       <c r="G23" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J23" s="55" t="s">
-        <v>46</v>
+      <c r="H23" s="52">
+        <v>1.4</v>
+      </c>
+      <c r="I23" s="52">
+        <v>1.4</v>
+      </c>
+      <c r="J23" s="55">
+        <v>1.4</v>
       </c>
       <c r="K23" s="52" t="s">
         <v>3</v>
@@ -3132,14 +3132,14 @@
       <c r="G24" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" s="55" t="s">
-        <v>46</v>
+      <c r="H24" s="52">
+        <v>1.48</v>
+      </c>
+      <c r="I24" s="52">
+        <v>1.48</v>
+      </c>
+      <c r="J24" s="55">
+        <v>1.48</v>
       </c>
       <c r="K24" s="52" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-02T08:50Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{7A3B7AEA-B3E3-4187-8138-5DF472694495}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{4929188C-61BE-4200-ADB0-87E62196A05F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46295</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>122357</v>
+        <v>137372</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>21994</v>
+        <v>22583</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>100363</v>
+        <v>114789</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2579,13 +2579,13 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="I11" s="36">
-        <v>1.2290000000000001</v>
+        <v>1.28</v>
       </c>
       <c r="J11" s="39">
-        <v>1.226</v>
+        <v>1.2270000000000001</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2637,10 +2637,10 @@
         <v>1.28</v>
       </c>
       <c r="L12" s="43">
-        <v>1.38</v>
+        <v>1.28</v>
       </c>
       <c r="M12" s="45">
-        <v>1.365</v>
+        <v>1.28</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>45179</v>
+        <v>53550</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2813,14 +2813,14 @@
       <c r="J16" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M16" s="54" t="s">
-        <v>46</v>
+      <c r="K16" s="52">
+        <v>1.22</v>
+      </c>
+      <c r="L16" s="52">
+        <v>1.22</v>
+      </c>
+      <c r="M16" s="54">
+        <v>1.22</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="39.9" customHeight="1">
@@ -2896,13 +2896,13 @@
         <v>46</v>
       </c>
       <c r="K18" s="58">
-        <v>1.2250000000000001</v>
+        <v>1.2330000000000001</v>
       </c>
       <c r="L18" s="58">
-        <v>1.2250000000000001</v>
+        <v>1.2330000000000001</v>
       </c>
       <c r="M18" s="60">
-        <v>1.2250000000000001</v>
+        <v>1.2330000000000001</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.22</v>
+        <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.232</v>
+        <v>1.31</v>
       </c>
       <c r="M19" s="45">
-        <v>1.2250000000000001</v>
+        <v>1.2589999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="54" t="s">
-        <v>46</v>
+      <c r="K20" s="52">
+        <v>1.3</v>
+      </c>
+      <c r="L20" s="52">
+        <v>1.38</v>
+      </c>
+      <c r="M20" s="54">
+        <v>1.3480000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3050,23 +3050,23 @@
       <c r="G22" s="67" t="s">
         <v>46</v>
       </c>
-      <c r="H22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="I22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="J22" s="68" t="s">
-        <v>46</v>
+      <c r="H22" s="65">
+        <v>1.31</v>
+      </c>
+      <c r="I22" s="65">
+        <v>1.65</v>
+      </c>
+      <c r="J22" s="68">
+        <v>1.363</v>
       </c>
       <c r="K22" s="65">
-        <v>1.24</v>
+        <v>1.2829999999999999</v>
       </c>
       <c r="L22" s="65">
-        <v>1.37</v>
+        <v>1.35</v>
       </c>
       <c r="M22" s="67">
-        <v>1.3320000000000001</v>
+        <v>1.3280000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3091,14 +3091,14 @@
       <c r="G23" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H23" s="52">
-        <v>1.4</v>
-      </c>
-      <c r="I23" s="52">
-        <v>1.4</v>
-      </c>
-      <c r="J23" s="55">
-        <v>1.4</v>
+      <c r="H23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J23" s="55" t="s">
+        <v>46</v>
       </c>
       <c r="K23" s="52" t="s">
         <v>3</v>
@@ -3132,23 +3132,23 @@
       <c r="G24" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="52">
-        <v>1.48</v>
-      </c>
-      <c r="I24" s="52">
-        <v>1.48</v>
-      </c>
-      <c r="J24" s="55">
-        <v>1.48</v>
-      </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="H24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="55" t="s">
+        <v>46</v>
+      </c>
+      <c r="K24" s="52">
+        <v>1.5</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.5</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.5</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-05T09:28Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{4929188C-61BE-4200-ADB0-87E62196A05F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{FC0515AD-1EE7-45E4-8557-B895DFF40958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46296</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>137372</v>
+        <v>136849</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22583</v>
+        <v>21870</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>114789</v>
+        <v>114979</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,7 +2582,7 @@
         <v>1.2</v>
       </c>
       <c r="I11" s="36">
-        <v>1.28</v>
+        <v>1.2290000000000001</v>
       </c>
       <c r="J11" s="39">
         <v>1.2270000000000001</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43">
-        <v>1.28</v>
-      </c>
-      <c r="L12" s="43">
-        <v>1.28</v>
-      </c>
-      <c r="M12" s="45">
-        <v>1.28</v>
+      <c r="K12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M12" s="45" t="s">
+        <v>46</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>53550</v>
+        <v>52020</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2813,14 +2813,14 @@
       <c r="J16" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K16" s="52">
-        <v>1.22</v>
-      </c>
-      <c r="L16" s="52">
-        <v>1.22</v>
-      </c>
-      <c r="M16" s="54">
-        <v>1.22</v>
+      <c r="K16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M16" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58">
-        <v>1.2330000000000001</v>
-      </c>
-      <c r="L18" s="58">
-        <v>1.2330000000000001</v>
-      </c>
-      <c r="M18" s="60">
-        <v>1.2330000000000001</v>
+      <c r="K18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.2250000000000001</v>
+        <v>1.36</v>
       </c>
       <c r="L19" s="43">
-        <v>1.31</v>
+        <v>1.36</v>
       </c>
       <c r="M19" s="45">
-        <v>1.2589999999999999</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.3</v>
+        <v>1.2330000000000001</v>
       </c>
       <c r="L20" s="52">
-        <v>1.38</v>
+        <v>1.234</v>
       </c>
       <c r="M20" s="54">
-        <v>1.3480000000000001</v>
+        <v>1.2330000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3051,22 +3051,22 @@
         <v>46</v>
       </c>
       <c r="H22" s="65">
-        <v>1.31</v>
+        <v>1.35</v>
       </c>
       <c r="I22" s="65">
-        <v>1.65</v>
+        <v>1.35</v>
       </c>
       <c r="J22" s="68">
-        <v>1.363</v>
+        <v>1.35</v>
       </c>
       <c r="K22" s="65">
-        <v>1.2829999999999999</v>
+        <v>1.3</v>
       </c>
       <c r="L22" s="65">
-        <v>1.35</v>
+        <v>1.52</v>
       </c>
       <c r="M22" s="67">
-        <v>1.3280000000000001</v>
+        <v>1.3839999999999999</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3100,14 +3100,14 @@
       <c r="J23" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M23" s="54" t="s">
-        <v>46</v>
+      <c r="K23" s="52">
+        <v>1.38</v>
+      </c>
+      <c r="L23" s="52">
+        <v>1.38</v>
+      </c>
+      <c r="M23" s="54">
+        <v>1.38</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.5</v>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-06T09:14Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{FC0515AD-1EE7-45E4-8557-B895DFF40958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{F8A15822-2750-434B-BD2F-828B91BAEED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46297</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>136849</v>
+        <v>140393</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>21870</v>
+        <v>23553</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>114979</v>
+        <v>116840</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,7 +2582,7 @@
         <v>1.2</v>
       </c>
       <c r="I11" s="36">
-        <v>1.2290000000000001</v>
+        <v>1.28</v>
       </c>
       <c r="J11" s="39">
         <v>1.2270000000000001</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>52020</v>
+        <v>52061</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2772,14 +2772,14 @@
       <c r="J15" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K15" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L15" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M15" s="54" t="s">
-        <v>46</v>
+      <c r="K15" s="52">
+        <v>1.35</v>
+      </c>
+      <c r="L15" s="52">
+        <v>1.35</v>
+      </c>
+      <c r="M15" s="54">
+        <v>1.35</v>
       </c>
     </row>
     <row r="16" spans="1:19" ht="39.9" customHeight="1">
@@ -2804,14 +2804,14 @@
       <c r="G16" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J16" s="55" t="s">
-        <v>46</v>
+      <c r="H16" s="52">
+        <v>1.22</v>
+      </c>
+      <c r="I16" s="52">
+        <v>1.22</v>
+      </c>
+      <c r="J16" s="55">
+        <v>1.22</v>
       </c>
       <c r="K16" s="52" t="s">
         <v>3</v>
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.36</v>
+        <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.36</v>
+        <v>1.31</v>
       </c>
       <c r="M19" s="45">
-        <v>1.36</v>
+        <v>1.25</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.2330000000000001</v>
+        <v>1.2270000000000001</v>
       </c>
       <c r="L20" s="52">
-        <v>1.234</v>
+        <v>1.2310000000000001</v>
       </c>
       <c r="M20" s="54">
-        <v>1.2330000000000001</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3050,23 +3050,23 @@
       <c r="G22" s="67" t="s">
         <v>46</v>
       </c>
-      <c r="H22" s="65">
-        <v>1.35</v>
-      </c>
-      <c r="I22" s="65">
-        <v>1.35</v>
-      </c>
-      <c r="J22" s="68">
-        <v>1.35</v>
-      </c>
-      <c r="K22" s="65">
-        <v>1.3</v>
-      </c>
-      <c r="L22" s="65">
-        <v>1.52</v>
-      </c>
-      <c r="M22" s="67">
-        <v>1.3839999999999999</v>
+      <c r="H22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="I22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="J22" s="68" t="s">
+        <v>46</v>
+      </c>
+      <c r="K22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="M22" s="67" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3100,14 +3100,14 @@
       <c r="J23" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="52">
-        <v>1.38</v>
-      </c>
-      <c r="L23" s="52">
-        <v>1.38</v>
-      </c>
-      <c r="M23" s="54">
-        <v>1.38</v>
+      <c r="K23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M23" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="K24" s="52">
+        <v>1.5</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.52</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.5069999999999999</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-07T09:04Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{F8A15822-2750-434B-BD2F-828B91BAEED3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{565E6186-B0F5-4C90-ADF5-7827C486E01D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46300</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>140393</v>
+        <v>137351</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23553</v>
+        <v>22897</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>116840</v>
+        <v>114454</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>52061</v>
+        <v>50115</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2772,14 +2772,14 @@
       <c r="J15" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K15" s="52">
-        <v>1.35</v>
-      </c>
-      <c r="L15" s="52">
-        <v>1.35</v>
-      </c>
-      <c r="M15" s="54">
-        <v>1.35</v>
+      <c r="K15" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L15" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M15" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="16" spans="1:19" ht="39.9" customHeight="1">
@@ -2804,14 +2804,14 @@
       <c r="G16" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="52">
-        <v>1.22</v>
-      </c>
-      <c r="I16" s="52">
-        <v>1.22</v>
-      </c>
-      <c r="J16" s="55">
-        <v>1.22</v>
+      <c r="H16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J16" s="55" t="s">
+        <v>46</v>
       </c>
       <c r="K16" s="52" t="s">
         <v>3</v>
@@ -2940,10 +2940,10 @@
         <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.31</v>
+        <v>1.35</v>
       </c>
       <c r="M19" s="45">
-        <v>1.25</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.2270000000000001</v>
+        <v>1.228</v>
       </c>
       <c r="L20" s="52">
-        <v>1.2310000000000001</v>
+        <v>1.228</v>
       </c>
       <c r="M20" s="54">
-        <v>1.23</v>
+        <v>1.228</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="L22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="M22" s="67" t="s">
-        <v>46</v>
+      <c r="K22" s="65">
+        <v>1.335</v>
+      </c>
+      <c r="L22" s="65">
+        <v>1.35</v>
+      </c>
+      <c r="M22" s="67">
+        <v>1.343</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3145,10 +3145,10 @@
         <v>1.5</v>
       </c>
       <c r="L24" s="52">
-        <v>1.52</v>
+        <v>1.5</v>
       </c>
       <c r="M24" s="54">
-        <v>1.5069999999999999</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-08T09:19Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{565E6186-B0F5-4C90-ADF5-7827C486E01D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{4305D642-EFE4-4F30-A322-29C7125A9314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46301</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>137351</v>
+        <v>140485</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22897</v>
+        <v>22996</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>114454</v>
+        <v>117489</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>50115</v>
+        <v>52215</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="60" t="s">
-        <v>46</v>
+      <c r="K18" s="58">
+        <v>1.2310000000000001</v>
+      </c>
+      <c r="L18" s="58">
+        <v>1.25</v>
+      </c>
+      <c r="M18" s="60">
+        <v>1.238</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2940,10 +2940,10 @@
         <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.35</v>
+        <v>1.288</v>
       </c>
       <c r="M19" s="45">
-        <v>1.23</v>
+        <v>1.236</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.228</v>
+        <v>1.232</v>
       </c>
       <c r="L20" s="52">
-        <v>1.228</v>
+        <v>1.33</v>
       </c>
       <c r="M20" s="54">
-        <v>1.228</v>
+        <v>1.2649999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3018,14 +3018,14 @@
       <c r="J21" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L21" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M21" s="60" t="s">
-        <v>46</v>
+      <c r="K21" s="58">
+        <v>1.32</v>
+      </c>
+      <c r="L21" s="58">
+        <v>1.32</v>
+      </c>
+      <c r="M21" s="60">
+        <v>1.32</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.335</v>
+        <v>1.4</v>
       </c>
       <c r="L22" s="65">
-        <v>1.35</v>
+        <v>1.4</v>
       </c>
       <c r="M22" s="67">
-        <v>1.343</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-09T03:34Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{4305D642-EFE4-4F30-A322-29C7125A9314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6F1ABE0B-EDF1-4E21-A769-13D08AEA2E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46302</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>140485</v>
+        <v>140450</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22996</v>
+        <v>23333</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>117489</v>
+        <v>117117</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2585,7 +2585,7 @@
         <v>1.28</v>
       </c>
       <c r="J11" s="39">
-        <v>1.2270000000000001</v>
+        <v>1.228</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>52215</v>
+        <v>49383</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2896,13 +2896,13 @@
         <v>46</v>
       </c>
       <c r="K18" s="58">
-        <v>1.2310000000000001</v>
+        <v>1.2250000000000001</v>
       </c>
       <c r="L18" s="58">
-        <v>1.25</v>
+        <v>1.35</v>
       </c>
       <c r="M18" s="60">
-        <v>1.238</v>
+        <v>1.323</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2940,10 +2940,10 @@
         <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.288</v>
+        <v>1.31</v>
       </c>
       <c r="M19" s="45">
-        <v>1.236</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52">
-        <v>1.232</v>
-      </c>
-      <c r="L20" s="52">
-        <v>1.33</v>
-      </c>
-      <c r="M20" s="54">
-        <v>1.2649999999999999</v>
+      <c r="K20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3018,14 +3018,14 @@
       <c r="J21" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K21" s="58">
-        <v>1.32</v>
-      </c>
-      <c r="L21" s="58">
-        <v>1.32</v>
-      </c>
-      <c r="M21" s="60">
-        <v>1.32</v>
+      <c r="K21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L21" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M21" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="L22" s="65">
-        <v>1.4</v>
+        <v>1.32</v>
       </c>
       <c r="M22" s="67">
-        <v>1.4</v>
+        <v>1.3160000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.5</v>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-13T02:33Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6F1ABE0B-EDF1-4E21-A769-13D08AEA2E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{DBFA1458-A844-47CE-85FE-60C21E2F57BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>140450</v>
+        <v>138364</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23333</v>
+        <v>22857</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>117117</v>
+        <v>115507</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2579,13 +2579,13 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>1.2</v>
+        <v>1.19</v>
       </c>
       <c r="I11" s="36">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="J11" s="39">
-        <v>1.228</v>
+        <v>1.2270000000000001</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>49383</v>
+        <v>48068</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58">
-        <v>1.2250000000000001</v>
-      </c>
-      <c r="L18" s="58">
-        <v>1.35</v>
-      </c>
-      <c r="M18" s="60">
-        <v>1.323</v>
+      <c r="K18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.2250000000000001</v>
+        <v>1.226</v>
       </c>
       <c r="L19" s="43">
         <v>1.31</v>
       </c>
       <c r="M19" s="45">
-        <v>1.23</v>
+        <v>1.2390000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="54" t="s">
-        <v>46</v>
+      <c r="K20" s="52">
+        <v>1.2310000000000001</v>
+      </c>
+      <c r="L20" s="52">
+        <v>1.2310000000000001</v>
+      </c>
+      <c r="M20" s="54">
+        <v>1.2310000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.3</v>
+        <v>1.35</v>
       </c>
       <c r="L22" s="65">
-        <v>1.32</v>
+        <v>1.35</v>
       </c>
       <c r="M22" s="67">
-        <v>1.3160000000000001</v>
+        <v>1.35</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="K24" s="52">
+        <v>1.5</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.5</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.5</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-14T04:47Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{DBFA1458-A844-47CE-85FE-60C21E2F57BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{6D54D01D-37CA-4B68-ADDA-7A891378F266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46304</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>138364</v>
+        <v>138749</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22857</v>
+        <v>23060</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>115507</v>
+        <v>115689</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2579,13 +2579,13 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>1.19</v>
+        <v>1.2</v>
       </c>
       <c r="I11" s="36">
-        <v>1.25</v>
+        <v>1.28</v>
       </c>
       <c r="J11" s="39">
-        <v>1.2270000000000001</v>
+        <v>1.228</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>48068</v>
+        <v>47425</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
+        <v>1.2250000000000001</v>
+      </c>
+      <c r="L19" s="43">
+        <v>1.23</v>
+      </c>
+      <c r="M19" s="45">
         <v>1.226</v>
-      </c>
-      <c r="L19" s="43">
-        <v>1.31</v>
-      </c>
-      <c r="M19" s="45">
-        <v>1.2390000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.2310000000000001</v>
+        <v>1.31</v>
       </c>
       <c r="L20" s="52">
-        <v>1.2310000000000001</v>
+        <v>1.35</v>
       </c>
       <c r="M20" s="54">
-        <v>1.2310000000000001</v>
+        <v>1.333</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65">
-        <v>1.35</v>
-      </c>
-      <c r="L22" s="65">
-        <v>1.35</v>
-      </c>
-      <c r="M22" s="67">
-        <v>1.35</v>
+      <c r="K22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="M22" s="67" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3100,14 +3100,14 @@
       <c r="J23" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L23" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M23" s="54" t="s">
-        <v>46</v>
+      <c r="K23" s="52">
+        <v>1.4</v>
+      </c>
+      <c r="L23" s="52">
+        <v>1.4</v>
+      </c>
+      <c r="M23" s="54">
+        <v>1.4</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.5</v>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-15T05:01Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{6D54D01D-37CA-4B68-ADDA-7A891378F266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{F2FB10A1-06FC-4603-8EE5-8824A253AF18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>138749</v>
+        <v>135189</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23060</v>
+        <v>22677</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>115689</v>
+        <v>112512</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>47425</v>
+        <v>44258</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="60" t="s">
-        <v>46</v>
+      <c r="K18" s="58">
+        <v>1.35</v>
+      </c>
+      <c r="L18" s="58">
+        <v>1.35</v>
+      </c>
+      <c r="M18" s="60">
+        <v>1.35</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2940,7 +2940,7 @@
         <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.23</v>
+        <v>1.2350000000000001</v>
       </c>
       <c r="M19" s="45">
         <v>1.226</v>
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.31</v>
+        <v>1.2290000000000001</v>
       </c>
       <c r="L20" s="52">
-        <v>1.35</v>
+        <v>1.232</v>
       </c>
       <c r="M20" s="54">
-        <v>1.333</v>
+        <v>1.2310000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="L22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="M22" s="67" t="s">
-        <v>46</v>
+      <c r="K22" s="65">
+        <v>1.32</v>
+      </c>
+      <c r="L22" s="65">
+        <v>1.43</v>
+      </c>
+      <c r="M22" s="67">
+        <v>1.373</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3100,14 +3100,14 @@
       <c r="J23" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K23" s="52">
-        <v>1.4</v>
-      </c>
-      <c r="L23" s="52">
-        <v>1.4</v>
-      </c>
-      <c r="M23" s="54">
-        <v>1.4</v>
+      <c r="K23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L23" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M23" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="K24" s="52">
+        <v>1.5</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.51</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.5049999999999999</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-16T03:04Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{F2FB10A1-06FC-4603-8EE5-8824A253AF18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{0B998D79-DA70-4491-9094-ADB099D81C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>135189</v>
+        <v>134160</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22677</v>
+        <v>22498</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>112512</v>
+        <v>111662</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>44258</v>
+        <v>43468</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2731,14 +2731,14 @@
       <c r="J14" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K14" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L14" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M14" s="45" t="s">
-        <v>46</v>
+      <c r="K14" s="43">
+        <v>1.3</v>
+      </c>
+      <c r="L14" s="43">
+        <v>1.3</v>
+      </c>
+      <c r="M14" s="45">
+        <v>1.3</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58">
-        <v>1.35</v>
-      </c>
-      <c r="L18" s="58">
-        <v>1.35</v>
-      </c>
-      <c r="M18" s="60">
-        <v>1.35</v>
+      <c r="K18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2940,10 +2940,10 @@
         <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.2350000000000001</v>
+        <v>1.31</v>
       </c>
       <c r="M19" s="45">
-        <v>1.226</v>
+        <v>1.23</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2968,23 +2968,23 @@
       <c r="G20" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J20" s="55" t="s">
-        <v>46</v>
+      <c r="H20" s="52">
+        <v>1.31</v>
+      </c>
+      <c r="I20" s="52">
+        <v>1.31</v>
+      </c>
+      <c r="J20" s="55">
+        <v>1.31</v>
       </c>
       <c r="K20" s="52">
-        <v>1.2290000000000001</v>
+        <v>1.288</v>
       </c>
       <c r="L20" s="52">
-        <v>1.232</v>
+        <v>1.36</v>
       </c>
       <c r="M20" s="54">
-        <v>1.2310000000000001</v>
+        <v>1.3149999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65">
-        <v>1.32</v>
-      </c>
-      <c r="L22" s="65">
-        <v>1.43</v>
-      </c>
-      <c r="M22" s="67">
-        <v>1.373</v>
+      <c r="K22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="M22" s="67" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3142,13 +3142,13 @@
         <v>46</v>
       </c>
       <c r="K24" s="52">
+        <v>1.48</v>
+      </c>
+      <c r="L24" s="52">
         <v>1.5</v>
       </c>
-      <c r="L24" s="52">
-        <v>1.51</v>
-      </c>
       <c r="M24" s="54">
-        <v>1.5049999999999999</v>
+        <v>1.484</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-19T02:33Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{0B998D79-DA70-4491-9094-ADB099D81C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{2D9C412D-F8E1-45E2-8312-6D5885A524AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46310</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>134160</v>
+        <v>130232</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22498</v>
+        <v>22777</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>111662</v>
+        <v>107455</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,10 +2582,10 @@
         <v>1.2</v>
       </c>
       <c r="I11" s="36">
-        <v>1.28</v>
+        <v>1.25</v>
       </c>
       <c r="J11" s="39">
-        <v>1.228</v>
+        <v>1.2270000000000001</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>43468</v>
+        <v>39991</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2731,14 +2731,14 @@
       <c r="J14" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K14" s="43">
-        <v>1.3</v>
-      </c>
-      <c r="L14" s="43">
-        <v>1.3</v>
-      </c>
-      <c r="M14" s="45">
-        <v>1.3</v>
+      <c r="K14" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L14" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M14" s="45" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="39.9" customHeight="1">
@@ -2940,10 +2940,10 @@
         <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.31</v>
+        <v>1.36</v>
       </c>
       <c r="M19" s="45">
-        <v>1.23</v>
+        <v>1.2669999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2968,23 +2968,23 @@
       <c r="G20" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H20" s="52">
-        <v>1.31</v>
-      </c>
-      <c r="I20" s="52">
-        <v>1.31</v>
-      </c>
-      <c r="J20" s="55">
-        <v>1.31</v>
+      <c r="H20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J20" s="55" t="s">
+        <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.288</v>
+        <v>1.3</v>
       </c>
       <c r="L20" s="52">
-        <v>1.36</v>
+        <v>1.37</v>
       </c>
       <c r="M20" s="54">
-        <v>1.3149999999999999</v>
+        <v>1.343</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52">
-        <v>1.48</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.5</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.484</v>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-20T07:50Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{2D9C412D-F8E1-45E2-8312-6D5885A524AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{D90D12B1-4BB8-442D-98E3-A2612477CEFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46311</v>
+        <v>46314</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>130232</v>
+        <v>128555</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22777</v>
+        <v>23964</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>107455</v>
+        <v>104591</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2579,7 +2579,7 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>1.2</v>
+        <v>1.2010000000000001</v>
       </c>
       <c r="I11" s="36">
         <v>1.25</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>39991</v>
+        <v>35307</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2804,14 +2804,14 @@
       <c r="G16" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J16" s="55" t="s">
-        <v>46</v>
+      <c r="H16" s="52">
+        <v>1.22</v>
+      </c>
+      <c r="I16" s="52">
+        <v>1.22</v>
+      </c>
+      <c r="J16" s="55">
+        <v>1.22</v>
       </c>
       <c r="K16" s="52" t="s">
         <v>3</v>
@@ -2940,10 +2940,10 @@
         <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.36</v>
+        <v>1.2310000000000001</v>
       </c>
       <c r="M19" s="45">
-        <v>1.2669999999999999</v>
+        <v>1.226</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52">
-        <v>1.3</v>
-      </c>
-      <c r="L20" s="52">
-        <v>1.37</v>
-      </c>
-      <c r="M20" s="54">
-        <v>1.343</v>
+      <c r="K20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-21T05:01Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{D90D12B1-4BB8-442D-98E3-A2612477CEFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{D098B3B1-F0D5-4BF5-B4E6-BAF436690AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46314</v>
+        <v>46315</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46314</v>
+        <v>46315</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>128555</v>
+        <v>129863</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23964</v>
+        <v>24172</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>104591</v>
+        <v>105691</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,10 +2582,10 @@
         <v>1.2010000000000001</v>
       </c>
       <c r="I11" s="36">
-        <v>1.25</v>
+        <v>1.28</v>
       </c>
       <c r="J11" s="39">
-        <v>1.2270000000000001</v>
+        <v>1.228</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M12" s="45" t="s">
-        <v>46</v>
+      <c r="K12" s="43">
+        <v>1.2150000000000001</v>
+      </c>
+      <c r="L12" s="43">
+        <v>1.2150000000000001</v>
+      </c>
+      <c r="M12" s="45">
+        <v>1.2150000000000001</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>35307</v>
+        <v>36777</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2763,14 +2763,14 @@
       <c r="G15" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H15" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I15" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J15" s="55" t="s">
-        <v>46</v>
+      <c r="H15" s="52">
+        <v>1.28</v>
+      </c>
+      <c r="I15" s="52">
+        <v>1.28</v>
+      </c>
+      <c r="J15" s="55">
+        <v>1.28</v>
       </c>
       <c r="K15" s="52" t="s">
         <v>3</v>
@@ -2804,14 +2804,14 @@
       <c r="G16" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H16" s="52">
-        <v>1.22</v>
-      </c>
-      <c r="I16" s="52">
-        <v>1.22</v>
-      </c>
-      <c r="J16" s="55">
-        <v>1.22</v>
+      <c r="H16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J16" s="55" t="s">
+        <v>46</v>
       </c>
       <c r="K16" s="52" t="s">
         <v>3</v>
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="60" t="s">
-        <v>46</v>
+      <c r="K18" s="58">
+        <v>1.35</v>
+      </c>
+      <c r="L18" s="58">
+        <v>1.35</v>
+      </c>
+      <c r="M18" s="60">
+        <v>1.35</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2940,10 +2940,10 @@
         <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.2310000000000001</v>
+        <v>1.31</v>
       </c>
       <c r="M19" s="45">
-        <v>1.226</v>
+        <v>1.232</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="54" t="s">
-        <v>46</v>
+      <c r="K20" s="52">
+        <v>1.228</v>
+      </c>
+      <c r="L20" s="52">
+        <v>1.29</v>
+      </c>
+      <c r="M20" s="54">
+        <v>1.23</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="K24" s="52">
+        <v>1.51</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.52</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.5129999999999999</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-22T02:47Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{D098B3B1-F0D5-4BF5-B4E6-BAF436690AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{34ECAFA4-E469-477E-A6A5-13C6D8584E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46315</v>
+        <v>46316</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>129863</v>
+        <v>129281</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>24172</v>
+        <v>23753</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>105691</v>
+        <v>105528</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2585,7 +2585,7 @@
         <v>1.28</v>
       </c>
       <c r="J11" s="39">
-        <v>1.228</v>
+        <v>1.2270000000000001</v>
       </c>
       <c r="K11" s="36" t="s">
         <v>50</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43">
-        <v>1.2150000000000001</v>
-      </c>
-      <c r="L12" s="43">
-        <v>1.2150000000000001</v>
-      </c>
-      <c r="M12" s="45">
-        <v>1.2150000000000001</v>
+      <c r="K12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L12" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M12" s="45" t="s">
+        <v>46</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>36777</v>
+        <v>36309</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2763,14 +2763,14 @@
       <c r="G15" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H15" s="52">
-        <v>1.28</v>
-      </c>
-      <c r="I15" s="52">
-        <v>1.28</v>
-      </c>
-      <c r="J15" s="55">
-        <v>1.28</v>
+      <c r="H15" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I15" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J15" s="55" t="s">
+        <v>46</v>
       </c>
       <c r="K15" s="52" t="s">
         <v>3</v>
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58">
-        <v>1.35</v>
-      </c>
-      <c r="L18" s="58">
-        <v>1.35</v>
-      </c>
-      <c r="M18" s="60">
-        <v>1.35</v>
+      <c r="K18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.2250000000000001</v>
+        <v>1.226</v>
       </c>
       <c r="L19" s="43">
-        <v>1.31</v>
+        <v>1.25</v>
       </c>
       <c r="M19" s="45">
-        <v>1.232</v>
+        <v>1.228</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.228</v>
+        <v>1.31</v>
       </c>
       <c r="L20" s="52">
-        <v>1.29</v>
+        <v>1.33</v>
       </c>
       <c r="M20" s="54">
-        <v>1.23</v>
+        <v>1.32</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3142,13 +3142,13 @@
         <v>46</v>
       </c>
       <c r="K24" s="52">
-        <v>1.51</v>
+        <v>1.5</v>
       </c>
       <c r="L24" s="52">
-        <v>1.52</v>
+        <v>1.55</v>
       </c>
       <c r="M24" s="54">
-        <v>1.5129999999999999</v>
+        <v>1.512</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-23T02:34Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{34ECAFA4-E469-477E-A6A5-13C6D8584E5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{8D729572-860B-4C22-A7D0-08FED0C12278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46316</v>
+        <v>46317</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>129281</v>
+        <v>126900</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23753</v>
+        <v>22837</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>105528</v>
+        <v>104063</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>36309</v>
+        <v>35534</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.226</v>
+        <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.25</v>
+        <v>1.31</v>
       </c>
       <c r="M19" s="45">
-        <v>1.228</v>
+        <v>1.232</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52">
-        <v>1.31</v>
-      </c>
-      <c r="L20" s="52">
-        <v>1.33</v>
-      </c>
-      <c r="M20" s="54">
-        <v>1.32</v>
+      <c r="K20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L20" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="L22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="M22" s="67" t="s">
-        <v>46</v>
+      <c r="K22" s="65">
+        <v>1.35</v>
+      </c>
+      <c r="L22" s="65">
+        <v>1.35</v>
+      </c>
+      <c r="M22" s="67">
+        <v>1.35</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3142,13 +3142,13 @@
         <v>46</v>
       </c>
       <c r="K24" s="52">
-        <v>1.5</v>
+        <v>1.55</v>
       </c>
       <c r="L24" s="52">
         <v>1.55</v>
       </c>
       <c r="M24" s="54">
-        <v>1.512</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-26T03:02Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{8D729572-860B-4C22-A7D0-08FED0C12278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{7F7733D0-81F5-42CE-A9C3-4E8A44D5DE60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46317</v>
+        <v>46318</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>126900</v>
+        <v>123899</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22837</v>
+        <v>22307</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>104063</v>
+        <v>101592</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2579,10 +2579,10 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>1.2010000000000001</v>
+        <v>1.2</v>
       </c>
       <c r="I11" s="36">
-        <v>1.28</v>
+        <v>1.228</v>
       </c>
       <c r="J11" s="39">
         <v>1.2270000000000001</v>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>35534</v>
+        <v>32893</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2940,10 +2940,10 @@
         <v>1.2250000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.31</v>
+        <v>1.36</v>
       </c>
       <c r="M19" s="45">
-        <v>1.232</v>
+        <v>1.2549999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2977,14 +2977,14 @@
       <c r="J20" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L20" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M20" s="54" t="s">
-        <v>46</v>
+      <c r="K20" s="52">
+        <v>1.37</v>
+      </c>
+      <c r="L20" s="52">
+        <v>1.37</v>
+      </c>
+      <c r="M20" s="54">
+        <v>1.37</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.35</v>
+        <v>1.33</v>
       </c>
       <c r="L22" s="65">
         <v>1.35</v>
       </c>
       <c r="M22" s="67">
-        <v>1.35</v>
+        <v>1.345</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3132,23 +3132,23 @@
       <c r="G24" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="I24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" s="55" t="s">
-        <v>46</v>
-      </c>
-      <c r="K24" s="52">
-        <v>1.55</v>
-      </c>
-      <c r="L24" s="52">
-        <v>1.55</v>
-      </c>
-      <c r="M24" s="54">
-        <v>1.55</v>
+      <c r="H24" s="52">
+        <v>1.52</v>
+      </c>
+      <c r="I24" s="52">
+        <v>1.52</v>
+      </c>
+      <c r="J24" s="55">
+        <v>1.52</v>
+      </c>
+      <c r="K24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M24" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-27T02:36Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{7F7733D0-81F5-42CE-A9C3-4E8A44D5DE60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{82A1D416-C1E4-448F-ACAE-EDF165F79E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46318</v>
+        <v>46321</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46318</v>
+        <v>46321</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>123899</v>
+        <v>124274</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22307</v>
+        <v>22686</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>101592</v>
+        <v>101588</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2579,7 +2579,7 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>1.2</v>
+        <v>1.202</v>
       </c>
       <c r="I11" s="36">
         <v>1.228</v>
@@ -2633,14 +2633,14 @@
       <c r="J12" s="46" t="s">
         <v>50</v>
       </c>
-      <c r="K12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L12" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M12" s="45" t="s">
-        <v>46</v>
+      <c r="K12" s="43">
+        <v>1.22</v>
+      </c>
+      <c r="L12" s="43">
+        <v>1.22</v>
+      </c>
+      <c r="M12" s="45">
+        <v>1.22</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>32893</v>
+        <v>33739</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="60" t="s">
-        <v>46</v>
+      <c r="K18" s="58">
+        <v>1.35</v>
+      </c>
+      <c r="L18" s="58">
+        <v>1.35</v>
+      </c>
+      <c r="M18" s="60">
+        <v>1.35</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2936,14 +2936,14 @@
       <c r="J19" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="43">
-        <v>1.2250000000000001</v>
-      </c>
-      <c r="L19" s="43">
-        <v>1.36</v>
-      </c>
-      <c r="M19" s="45">
-        <v>1.2549999999999999</v>
+      <c r="K19" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="L19" s="43" t="s">
+        <v>3</v>
+      </c>
+      <c r="M19" s="45" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.37</v>
+        <v>1.2250000000000001</v>
       </c>
       <c r="L20" s="52">
-        <v>1.37</v>
+        <v>1.2310000000000001</v>
       </c>
       <c r="M20" s="54">
-        <v>1.37</v>
+        <v>1.2290000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65">
-        <v>1.33</v>
-      </c>
-      <c r="L22" s="65">
-        <v>1.35</v>
-      </c>
-      <c r="M22" s="67">
-        <v>1.345</v>
+      <c r="K22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="L22" s="65" t="s">
+        <v>3</v>
+      </c>
+      <c r="M22" s="67" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3132,14 +3132,14 @@
       <c r="G24" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="H24" s="52">
-        <v>1.52</v>
-      </c>
-      <c r="I24" s="52">
-        <v>1.52</v>
-      </c>
-      <c r="J24" s="55">
-        <v>1.52</v>
+      <c r="H24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="I24" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="55" t="s">
+        <v>46</v>
       </c>
       <c r="K24" s="52" t="s">
         <v>3</v>
@@ -3182,14 +3182,14 @@
       <c r="J25" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K25" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L25" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M25" s="54" t="s">
-        <v>46</v>
+      <c r="K25" s="52">
+        <v>1.6</v>
+      </c>
+      <c r="L25" s="52">
+        <v>1.6</v>
+      </c>
+      <c r="M25" s="54">
+        <v>1.6</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-28T03:18Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{82A1D416-C1E4-448F-ACAE-EDF165F79E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{06799A2C-E819-4BDD-BE32-8DE835072BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46321</v>
+        <v>46322</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46321</v>
+        <v>46322</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>124274</v>
+        <v>124736</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>22686</v>
+        <v>23103</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>101588</v>
+        <v>101633</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,7 +2582,7 @@
         <v>1.202</v>
       </c>
       <c r="I11" s="36">
-        <v>1.228</v>
+        <v>1.28</v>
       </c>
       <c r="J11" s="39">
         <v>1.2270000000000001</v>
@@ -2634,13 +2634,13 @@
         <v>50</v>
       </c>
       <c r="K12" s="43">
-        <v>1.22</v>
+        <v>1.228</v>
       </c>
       <c r="L12" s="43">
-        <v>1.22</v>
+        <v>1.228</v>
       </c>
       <c r="M12" s="45">
-        <v>1.22</v>
+        <v>1.228</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>33739</v>
+        <v>33489</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2854,14 +2854,14 @@
       <c r="J17" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K17" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="54" t="s">
-        <v>46</v>
+      <c r="K17" s="52">
+        <v>1.29</v>
+      </c>
+      <c r="L17" s="52">
+        <v>1.29</v>
+      </c>
+      <c r="M17" s="54">
+        <v>1.29</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58">
-        <v>1.35</v>
-      </c>
-      <c r="L18" s="58">
-        <v>1.35</v>
-      </c>
-      <c r="M18" s="60">
-        <v>1.35</v>
+      <c r="K18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="L18" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="M18" s="60" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2936,14 +2936,14 @@
       <c r="J19" s="46" t="s">
         <v>46</v>
       </c>
-      <c r="K19" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="L19" s="43" t="s">
-        <v>3</v>
-      </c>
-      <c r="M19" s="45" t="s">
-        <v>46</v>
+      <c r="K19" s="43">
+        <v>1.2250000000000001</v>
+      </c>
+      <c r="L19" s="43">
+        <v>1.3</v>
+      </c>
+      <c r="M19" s="45">
+        <v>1.2709999999999999</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.2250000000000001</v>
+        <v>1.228</v>
       </c>
       <c r="L20" s="52">
-        <v>1.2310000000000001</v>
+        <v>1.355</v>
       </c>
       <c r="M20" s="54">
-        <v>1.2290000000000001</v>
+        <v>1.24</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3059,14 +3059,14 @@
       <c r="J22" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="L22" s="65" t="s">
-        <v>3</v>
-      </c>
-      <c r="M22" s="67" t="s">
-        <v>46</v>
+      <c r="K22" s="65">
+        <v>1.34</v>
+      </c>
+      <c r="L22" s="65">
+        <v>1.34</v>
+      </c>
+      <c r="M22" s="67">
+        <v>1.34</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3182,14 +3182,14 @@
       <c r="J25" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K25" s="52">
-        <v>1.6</v>
-      </c>
-      <c r="L25" s="52">
-        <v>1.6</v>
-      </c>
-      <c r="M25" s="54">
-        <v>1.6</v>
+      <c r="K25" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L25" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M25" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-29T02:37Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{06799A2C-E819-4BDD-BE32-8DE835072BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{57042BE6-FCFA-4CFF-9949-90350CAC04C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="51">
   <si>
     <t xml:space="preserve">Financial Markets Department </t>
     <phoneticPr fontId="4"/>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46322</v>
+        <v>46323</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46322</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>124736</v>
+        <v>123193</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>23103</v>
+        <v>21795</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>101633</v>
+        <v>101398</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2579,10 +2579,10 @@
         <v>50</v>
       </c>
       <c r="H11" s="36">
-        <v>1.202</v>
+        <v>1.2030000000000001</v>
       </c>
       <c r="I11" s="36">
-        <v>1.28</v>
+        <v>1.2749999999999999</v>
       </c>
       <c r="J11" s="39">
         <v>1.2270000000000001</v>
@@ -2634,13 +2634,13 @@
         <v>50</v>
       </c>
       <c r="K12" s="43">
-        <v>1.228</v>
+        <v>1.22</v>
       </c>
       <c r="L12" s="43">
-        <v>1.228</v>
+        <v>1.22</v>
       </c>
       <c r="M12" s="45">
-        <v>1.228</v>
+        <v>1.22</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>33489</v>
+        <v>33424</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2813,14 +2813,14 @@
       <c r="J16" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L16" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M16" s="54" t="s">
-        <v>46</v>
+      <c r="K16" s="52">
+        <v>1.28</v>
+      </c>
+      <c r="L16" s="52">
+        <v>1.28</v>
+      </c>
+      <c r="M16" s="54">
+        <v>1.28</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="39.9" customHeight="1">
@@ -2854,14 +2854,14 @@
       <c r="J17" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K17" s="52">
-        <v>1.29</v>
-      </c>
-      <c r="L17" s="52">
-        <v>1.29</v>
-      </c>
-      <c r="M17" s="54">
-        <v>1.29</v>
+      <c r="K17" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L17" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M17" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,10 +2937,10 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.2250000000000001</v>
+        <v>1.2310000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="M19" s="45">
         <v>1.2709999999999999</v>
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.228</v>
+        <v>1.31</v>
       </c>
       <c r="L20" s="52">
-        <v>1.355</v>
+        <v>1.31</v>
       </c>
       <c r="M20" s="54">
-        <v>1.24</v>
+        <v>1.31</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3141,14 +3141,14 @@
       <c r="J24" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L24" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M24" s="54" t="s">
-        <v>46</v>
+      <c r="K24" s="52">
+        <v>1.52</v>
+      </c>
+      <c r="L24" s="52">
+        <v>1.57</v>
+      </c>
+      <c r="M24" s="54">
+        <v>1.5409999999999999</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">
@@ -3182,14 +3182,14 @@
       <c r="J25" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K25" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L25" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M25" s="54" t="s">
-        <v>46</v>
+      <c r="K25" s="52">
+        <v>1.65</v>
+      </c>
+      <c r="L25" s="52">
+        <v>1.65</v>
+      </c>
+      <c r="M25" s="54">
+        <v>1.65</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>

<commit_message>
data(jpy): daily refresh 2026-10-30T02:32Z
</commit_message>
<xml_diff>
--- a/logs/jpy/raw/fcall.xlsx
+++ b/logs/jpy/raw/fcall.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{57042BE6-FCFA-4CFF-9949-90350CAC04C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{F6A0F8A1-2637-4256-8165-74800869CA1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2345,7 +2345,7 @@
   <sheetData>
     <row r="1" spans="1:19" ht="24.9" customHeight="1">
       <c r="A1" s="78">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1" s="80"/>
       <c r="K1" s="2"/>
@@ -2354,7 +2354,7 @@
       <c r="N1" s="3"/>
       <c r="R1" s="83"/>
       <c r="S1" s="84">
-        <v>46323</v>
+        <v>46324</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24.9" customHeight="1">
@@ -2473,7 +2473,7 @@
       <c r="Q8" s="90"/>
       <c r="R8" s="90"/>
       <c r="S8" s="17">
-        <v>123193</v>
+        <v>123946</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="39.9" customHeight="1">
@@ -2505,7 +2505,7 @@
       <c r="Q9" s="92"/>
       <c r="R9" s="92"/>
       <c r="S9" s="26">
-        <v>21795</v>
+        <v>21766</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="39.9" customHeight="1" thickBot="1">
@@ -2553,7 +2553,7 @@
       <c r="Q10" s="94"/>
       <c r="R10" s="94"/>
       <c r="S10" s="33">
-        <v>101398</v>
+        <v>102180</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="39.9" customHeight="1" thickTop="1">
@@ -2582,7 +2582,7 @@
         <v>1.2030000000000001</v>
       </c>
       <c r="I11" s="36">
-        <v>1.2749999999999999</v>
+        <v>1.228</v>
       </c>
       <c r="J11" s="39">
         <v>1.2270000000000001</v>
@@ -2634,13 +2634,13 @@
         <v>50</v>
       </c>
       <c r="K12" s="43">
-        <v>1.22</v>
+        <v>1.3</v>
       </c>
       <c r="L12" s="43">
-        <v>1.22</v>
+        <v>1.3</v>
       </c>
       <c r="M12" s="45">
-        <v>1.22</v>
+        <v>1.3</v>
       </c>
       <c r="O12" s="47"/>
       <c r="P12" s="48"/>
@@ -2697,7 +2697,7 @@
       <c r="Q13" s="87"/>
       <c r="R13" s="88"/>
       <c r="S13" s="49">
-        <v>33424</v>
+        <v>33386</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="39.9" customHeight="1">
@@ -2813,14 +2813,14 @@
       <c r="J16" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K16" s="52">
-        <v>1.28</v>
-      </c>
-      <c r="L16" s="52">
-        <v>1.28</v>
-      </c>
-      <c r="M16" s="54">
-        <v>1.28</v>
+      <c r="K16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L16" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M16" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="39.9" customHeight="1">
@@ -2854,14 +2854,14 @@
       <c r="J17" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K17" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="L17" s="52" t="s">
-        <v>3</v>
-      </c>
-      <c r="M17" s="54" t="s">
-        <v>46</v>
+      <c r="K17" s="52">
+        <v>1.2270000000000001</v>
+      </c>
+      <c r="L17" s="52">
+        <v>1.23</v>
+      </c>
+      <c r="M17" s="54">
+        <v>1.228</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="39.9" customHeight="1">
@@ -2895,14 +2895,14 @@
       <c r="J18" s="61" t="s">
         <v>46</v>
       </c>
-      <c r="K18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="L18" s="58" t="s">
-        <v>3</v>
-      </c>
-      <c r="M18" s="60" t="s">
-        <v>46</v>
+      <c r="K18" s="58">
+        <v>1.2789999999999999</v>
+      </c>
+      <c r="L18" s="58">
+        <v>1.2789999999999999</v>
+      </c>
+      <c r="M18" s="60">
+        <v>1.2789999999999999</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="39.9" customHeight="1">
@@ -2937,13 +2937,13 @@
         <v>46</v>
       </c>
       <c r="K19" s="43">
-        <v>1.2310000000000001</v>
+        <v>1.2270000000000001</v>
       </c>
       <c r="L19" s="43">
-        <v>1.34</v>
+        <v>1.31</v>
       </c>
       <c r="M19" s="45">
-        <v>1.2709999999999999</v>
+        <v>1.2390000000000001</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="39.9" customHeight="1">
@@ -2978,13 +2978,13 @@
         <v>46</v>
       </c>
       <c r="K20" s="52">
-        <v>1.31</v>
+        <v>1.228</v>
       </c>
       <c r="L20" s="52">
-        <v>1.31</v>
+        <v>1.36</v>
       </c>
       <c r="M20" s="54">
-        <v>1.31</v>
+        <v>1.268</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="39.9" customHeight="1">
@@ -3060,13 +3060,13 @@
         <v>46</v>
       </c>
       <c r="K22" s="65">
-        <v>1.34</v>
+        <v>1.29</v>
       </c>
       <c r="L22" s="65">
-        <v>1.34</v>
+        <v>1.65</v>
       </c>
       <c r="M22" s="67">
-        <v>1.34</v>
+        <v>1.3640000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:13" ht="39.9" customHeight="1">
@@ -3142,13 +3142,13 @@
         <v>46</v>
       </c>
       <c r="K24" s="52">
-        <v>1.52</v>
+        <v>1.55</v>
       </c>
       <c r="L24" s="52">
-        <v>1.57</v>
+        <v>1.55</v>
       </c>
       <c r="M24" s="54">
-        <v>1.5409999999999999</v>
+        <v>1.55</v>
       </c>
     </row>
     <row r="25" spans="1:13" ht="39.9" customHeight="1">
@@ -3182,14 +3182,14 @@
       <c r="J25" s="55" t="s">
         <v>46</v>
       </c>
-      <c r="K25" s="52">
-        <v>1.65</v>
-      </c>
-      <c r="L25" s="52">
-        <v>1.65</v>
-      </c>
-      <c r="M25" s="54">
-        <v>1.65</v>
+      <c r="K25" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="L25" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="M25" s="54" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:13" ht="39.9" customHeight="1">

</xml_diff>